<commit_message>
Round the rider to 90 000 and retitle the commission line
Technical rider goes to a round 90 000 ₽ in place of the estimate's exact
75 669 ₽, which carries the total to 228 000 ₽: costs 190 000 plus 38 000 of
commission. The estimate figure stays in the README as the source.

Line 4 is now "Комиссия и налоги" rather than "Комиссия сверху", and the
caption drops the orchestra and the street address — just "Концерт ·
20.10.2026 · Музей ЗИЛАРТ".

Adds the PNG of the table and the HTML it renders from; the notes block
under the table is gone at the client's request.

Recalculated: 6 formulas, 0 errors, totals checked independently.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RA1yrtrcqV5rmuM1iwZjp1
</commit_message>
<xml_diff>
--- a/event-zilart/Бюджет_ЗИЛАРТ_20.10.2026.xlsx
+++ b/event-zilart/Бюджет_ЗИЛАРТ_20.10.2026.xlsx
@@ -25,7 +25,7 @@
     <t xml:space="preserve">БЮДЖЕТ МЕРОПРИЯТИЯ</t>
   </si>
   <si>
-    <t xml:space="preserve">Оркестр, концерт · 20.10.2026 · Музей ЗИЛАРТ, бул. Братьев Весниных, 3 (3 этаж)</t>
+    <t xml:space="preserve">Концерт · 20.10.2026 · Музей ЗИЛАРТ</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Технический райдер (смета СМ-2026-024)</t>
   </si>
   <si>
-    <t xml:space="preserve">Спотыкач, 04.10.2026: позиции 68 790 ₽ + налог 10%</t>
+    <t xml:space="preserve">Округлённая сумма. По смете Спотыкача 75 669 ₽ (68 790 ₽ + налог 10%)</t>
   </si>
   <si>
     <t xml:space="preserve">Музыканты</t>
@@ -61,10 +61,10 @@
     <t xml:space="preserve">ИТОГО РАСХОДЫ</t>
   </si>
   <si>
-    <t xml:space="preserve">Комиссия сверху</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Начисляется на всю сумму расходов</t>
+    <t xml:space="preserve">Комиссия и налоги</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20% на всю сумму расходов</t>
   </si>
   <si>
     <t xml:space="preserve">ИТОГО К ОПЛАТЕ</t>
@@ -73,10 +73,10 @@
     <t xml:space="preserve">• Жёлтые ячейки — вводимые значения, остальное считается формулами.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Райдер взят итоговой суммой по смете СМ-2026-024 (налог 10% уже внутри).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Комиссия округлена до рубля: точное значение 35 133,80 ₽.</t>
+    <t xml:space="preserve">• Райдер округлён до 90 000 ₽; по смете СМ-2026-024 выходит 75 669 ₽ (налог 10% внутри).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Комиссия и налоги — 20% на всю сумму расходов.</t>
   </si>
   <si>
     <t xml:space="preserve">• Дата на уточнении — по примечанию в смете ожидается согласование с артистами после просмотра площадки.</t>
@@ -595,11 +595,11 @@
         <v>1</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>75669</v>
+        <v>90000</v>
       </c>
       <c r="E5" s="9" t="n">
         <f aca="false">C5*D5</f>
-        <v>75669</v>
+        <v>90000</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>8</v>
@@ -653,7 +653,7 @@
       <c r="D8" s="10"/>
       <c r="E8" s="12" t="n">
         <f aca="false">SUM(E5:E7)</f>
-        <v>175669</v>
+        <v>190000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -668,7 +668,7 @@
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">ROUND($E$8*D9,0)</f>
-        <v>35134</v>
+        <v>38000</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>14</v>
@@ -683,7 +683,7 @@
       <c r="D10" s="14"/>
       <c r="E10" s="16" t="n">
         <f aca="false">E8+E9</f>
-        <v>210803</v>
+        <v>228000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Source the rider line from the corrected rider
The budget line read "Технический райдер (смета СМ-2026-024)" while showing
90 000 ₽, but that estimate totals 75 669 ₽ — the citation contradicted the
figure. The line now just reads "Технический райдер" and takes its amount
from the corrected rider.

The original estimate PDF stays in the folder as history, and the README
says plainly that the budget no longer draws from it.

Adds shot.js, which renders budget.png from budget-card.html, so the image
can be rebuilt after a container reset.

Recalculated: 6 formulas, 0 errors, totals verified.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RA1yrtrcqV5rmuM1iwZjp1
</commit_message>
<xml_diff>
--- a/event-zilart/Бюджет_ЗИЛАРТ_20.10.2026.xlsx
+++ b/event-zilart/Бюджет_ЗИЛАРТ_20.10.2026.xlsx
@@ -43,10 +43,10 @@
     <t xml:space="preserve">Сумма, ₽</t>
   </si>
   <si>
-    <t xml:space="preserve">Технический райдер (смета СМ-2026-024)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Округлённая сумма. По смете Спотыкача 75 669 ₽ (68 790 ₽ + налог 10%)</t>
+    <t xml:space="preserve">Технический райдер</t>
+  </si>
+  <si>
+    <t xml:space="preserve">По скорректированному райдеру</t>
   </si>
   <si>
     <t xml:space="preserve">Музыканты</t>

</xml_diff>

<commit_message>
Take the rider from the 05.10 revision of the estimate
The corrected estimate CM-2026-024 came in at 79 536 ₽ — 72 305 ₽ of line
items plus the 10% tax — replacing the 90 000 ₽ placeholder. Total to pay
falls to 215 443 ₽: costs 179 536 plus 35 907 of commission.

Line items moved by +3 515 ₽ against the first revision: a fourth Sennheiser
IEM G4, one K&M stand fewer, an extra Dekko JR204, the Radial PRO48 dropped
for a DBX DJDI, and a stereo jack pair added. The README tabulates it and
both PDFs stay in the folder.

Recalculated: 6 formulas, 0 errors, totals verified independently.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RA1yrtrcqV5rmuM1iwZjp1
</commit_message>
<xml_diff>
--- a/event-zilart/Бюджет_ЗИЛАРТ_20.10.2026.xlsx
+++ b/event-zilart/Бюджет_ЗИЛАРТ_20.10.2026.xlsx
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Технический райдер</t>
   </si>
   <si>
-    <t xml:space="preserve">По скорректированному райдеру</t>
+    <t xml:space="preserve">Смета СМ-2026-024, ред. от 05.10.2026: 72 305 ₽ + налог 10%</t>
   </si>
   <si>
     <t xml:space="preserve">Музыканты</t>
@@ -73,7 +73,7 @@
     <t xml:space="preserve">• Жёлтые ячейки — вводимые значения, остальное считается формулами.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Райдер округлён до 90 000 ₽; по смете СМ-2026-024 выходит 75 669 ₽ (налог 10% внутри).</t>
+    <t xml:space="preserve">• Райдер — итог сметы СМ-2026-024 в редакции от 05.10.2026 (налог 10% внутри).</t>
   </si>
   <si>
     <t xml:space="preserve">• Комиссия и налоги — 20% на всю сумму расходов.</t>
@@ -595,11 +595,11 @@
         <v>1</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>90000</v>
+        <v>79536</v>
       </c>
       <c r="E5" s="9" t="n">
         <f aca="false">C5*D5</f>
-        <v>90000</v>
+        <v>79536</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>8</v>
@@ -653,7 +653,7 @@
       <c r="D8" s="10"/>
       <c r="E8" s="12" t="n">
         <f aca="false">SUM(E5:E7)</f>
-        <v>190000</v>
+        <v>179536</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -668,7 +668,7 @@
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">ROUND($E$8*D9,0)</f>
-        <v>38000</v>
+        <v>35907</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>14</v>
@@ -683,7 +683,7 @@
       <c r="D10" s="14"/>
       <c r="E10" s="16" t="n">
         <f aca="false">E8+E9</f>
-        <v>228000</v>
+        <v>215443</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>